<commit_message>
Update iPlanet Store Locator and database search
</commit_message>
<xml_diff>
--- a/Master Sheet.xlsx
+++ b/Master Sheet.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Documents\AI Work\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iPlanet AI Store Locator\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$82</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -24,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="593">
   <si>
     <t>Store Name</t>
   </si>
@@ -51,9 +54,6 @@
   </si>
   <si>
     <t>Google Maps / location</t>
-  </si>
-  <si>
-    <t>Latitude &amp; Longitude, if available</t>
   </si>
   <si>
     <t>iPlanet Pody Bazaar</t>
@@ -672,9 +672,6 @@
     <t>KNR 1</t>
   </si>
   <si>
-    <t>Keralam</t>
-  </si>
-  <si>
     <t>Kannur–Kuthuparamba Road, Thana, Near Lifestyle, Kannur – 670012</t>
   </si>
   <si>
@@ -876,10 +873,987 @@
     <t>12.9719° N / 77.6412° E</t>
   </si>
   <si>
-    <t xml:space="preserve">         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">iPlanet </t>
+    <t>iPlanet Dharamapuri</t>
+  </si>
+  <si>
+    <t>DPR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. 9/4, Salem Main Road, Indhira Nagar, Dharmapuri, Tamil Nadu – 636705 </t>
+  </si>
+  <si>
+    <t>MSK Mandapam</t>
+  </si>
+  <si>
+    <t>Salem Main Road, Indhira Nagar</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=9%2F4+Salem+Main+Road+Indhira+Nagar+Dharmapuri+636705</t>
+  </si>
+  <si>
+    <t>12.117410 / 78.155976</t>
+  </si>
+  <si>
+    <t>iPlanet Nexus Shantiniketan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NSN 1 </t>
+  </si>
+  <si>
+    <t>No. 4, Upper Ground Floor</t>
+  </si>
+  <si>
+    <t>Thigalarapalya</t>
+  </si>
+  <si>
+    <t>No. 4, Upper Ground Floor, Forum Mall, ITPL Main Road, near Thigalarapalya, Bengaluru – 560048.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Nexus+Shantiniketan+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.990 / 77.728</t>
+  </si>
+  <si>
+    <t>iPlanet Whitefield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRM 1 </t>
+  </si>
+  <si>
+    <t>No. 2, Upper Ground Floor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KAM 1 </t>
+  </si>
+  <si>
+    <t>iPlanet Kalyan Nagar</t>
+  </si>
+  <si>
+    <t>Kalyan Nagar</t>
+  </si>
+  <si>
+    <t>Sunshine Complex, near HRBR Layout</t>
+  </si>
+  <si>
+    <t>No. 5, Ground Floor, Sunshine Complex, 4th E Main Road, HRBR Layout 3rd Block, Kalyan Nagar, Bengaluru – 560043.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Sunshine+Complex+Kalyan+Nagar+Bengaluru</t>
+  </si>
+  <si>
+    <t>13.028 / 77.644</t>
+  </si>
+  <si>
+    <t>iPlanet Hennur</t>
+  </si>
+  <si>
+    <t>HNR 1</t>
+  </si>
+  <si>
+    <t>Near Ramdev Mart</t>
+  </si>
+  <si>
+    <t>Hennur Bagalur Main Road</t>
+  </si>
+  <si>
+    <t>No. 7, Ground Floor, Hennur Bagalur Main Road, Kothanur, Bengaluru – 560077.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Hennur+Bagalur+Main+Road+Kothanur+Bengaluru</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 13.0610 / 77.6480</t>
+  </si>
+  <si>
+    <t>Mahadevapura</t>
+  </si>
+  <si>
+    <t>No. 2, Upper Ground Floor, Whitefield Main Road, Devasandra Industrial Estate, Mahadevapura, Bengaluru – 560048.</t>
+  </si>
+  <si>
+    <t>12.991 / 77.7040</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Whitefield+Main+Road+Mahadevapura+Bengaluru</t>
+  </si>
+  <si>
+    <t>iPlanet Sahakara Nagar</t>
+  </si>
+  <si>
+    <t>SAH 1</t>
+  </si>
+  <si>
+    <t>Opposite McDonald's.</t>
+  </si>
+  <si>
+    <t>F Block, 60 Feet Road</t>
+  </si>
+  <si>
+    <t>No. 510, F Block, 60 Feet Road, Sahakara Nagar, Bengaluru – 560092.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+510+F+Block+Sahakara+Nagar+Bengaluru+560092</t>
+  </si>
+  <si>
+    <t>13.0620 / 77.5800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iPlanet Bell Road </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEL 1 </t>
+  </si>
+  <si>
+    <t>Opposite Ramaiah Hospital signal.</t>
+  </si>
+  <si>
+    <t>80 Feet Road, Devasandra Layout</t>
+  </si>
+  <si>
+    <t>No. 55/58, 80 Feet Road, Devasandra Layout, Bengaluru – 560094.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+55%2F58+80+Feet+Road+Devasandra+Layout+Bengaluru</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 13.0320 / 77.5700</t>
+  </si>
+  <si>
+    <t>iPlanet Yelahanka</t>
+  </si>
+  <si>
+    <t>YNK 1</t>
+  </si>
+  <si>
+    <t>1st A Main Road</t>
+  </si>
+  <si>
+    <t>Near Vasthra Fashion.</t>
+  </si>
+  <si>
+    <t>No. 38, 1st A Main Road, Yelahanka Satellite Town, near Vasthra Fashion, Bengaluru – 560064.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+38+1st+A+Main+Road+Yelahanka+Bengaluru</t>
+  </si>
+  <si>
+    <t>13.1000 / 77.5960</t>
+  </si>
+  <si>
+    <t>iPlanet JP Nagar</t>
+  </si>
+  <si>
+    <t>JPN 1</t>
+  </si>
+  <si>
+    <t>Puttenahalli Road</t>
+  </si>
+  <si>
+    <t>JP Nagar 7th Phase</t>
+  </si>
+  <si>
+    <t>Ground Floor, Puttenahalli Road, Ramaiah Garden, JP Nagar 7th Phase, Bengaluru – 560078.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/dir/?api=1&amp;destination=iPlanet+JP+Nagar+7th+Phase+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.906 / 77.5850</t>
+  </si>
+  <si>
+    <t>JNG 1</t>
+  </si>
+  <si>
+    <t>Murari Tower, Jayanagar 2nd Block</t>
+  </si>
+  <si>
+    <t>T. Mariappa Road</t>
+  </si>
+  <si>
+    <t>No. 27, Murari Tower, T. Mariappa Road, 2nd Block, Jayanagar, Bengaluru – 560011.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Murari+Tower+Jayanagar+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.9250 / 77.5830</t>
+  </si>
+  <si>
+    <t>RMM 1</t>
+  </si>
+  <si>
+    <t>Ground Floor, Royal Meenakshi Mall</t>
+  </si>
+  <si>
+    <t>Bannerghatta Road, Hulimavu</t>
+  </si>
+  <si>
+    <t>Ground Floor, Royal Meenakshi Mall, No. 424/376/487, Bannerghatta Road, Hulimavu, Bengaluru – 560076.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Royal+Meenakshi+Mall+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.8690 / 77.5980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSK 1 </t>
+  </si>
+  <si>
+    <t>iPlanet Banashankari</t>
+  </si>
+  <si>
+    <t>iPlanet Jayanagar</t>
+  </si>
+  <si>
+    <t>iPlanet Royal Meenakshi Mall</t>
+  </si>
+  <si>
+    <t>Opposite Smart Bazaar</t>
+  </si>
+  <si>
+    <t>No. 24, G.R. Pristine, 80 Feet Road, 3rd Phase, Banashankari 3rd Stage, Bengaluru – 560085.</t>
+  </si>
+  <si>
+    <t>3rd Phase, Banashankari 3rd Stage</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Banashankari+GR+Pristine+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.9250 / 77.5650</t>
+  </si>
+  <si>
+    <t>iPlanet Kengeri</t>
+  </si>
+  <si>
+    <t>KNG 1</t>
+  </si>
+  <si>
+    <t>Opposite Shivashakti Hospital</t>
+  </si>
+  <si>
+    <t>No. 16, Outer Ring Road, Nagadevanahalli Main Road, opposite Shivashakti Hospital, RR Layout, Bengaluru – 560056.</t>
+  </si>
+  <si>
+    <t>Outer Ring Road, Nagadevanahalli Main Road</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+16+Outer+Ring+Road+Nagadevanahalli+Bengaluru+560056</t>
+  </si>
+  <si>
+    <t>12.935772 /77.492358</t>
+  </si>
+  <si>
+    <t>iPlanet Forum Falcon City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FFC 1 </t>
+  </si>
+  <si>
+    <t>Near Anjanadri Layout and Konanakunte Cross Metro Station</t>
+  </si>
+  <si>
+    <t>Kanakapura Main Road</t>
+  </si>
+  <si>
+    <t>No. 1182, Kanakapura Main Road, Konanakunte, Bengaluru – 560062.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Forum+South+Konanakunte+Bengaluru</t>
+  </si>
+  <si>
+    <t>12.8830 / 77.5700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iPlanet Peenya </t>
+  </si>
+  <si>
+    <t>PNA 1</t>
+  </si>
+  <si>
+    <t>Hesaraghatta Road, Defence Colony</t>
+  </si>
+  <si>
+    <t>Beside Tanishq Jewellery.</t>
+  </si>
+  <si>
+    <t>No. 5, Shree Anjanadri, Hesaraghatta Road, Defence Colony, Nagasandra, Bengaluru – 560073</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Peenya+Shree+Anjanadri+Bengaluru</t>
+  </si>
+  <si>
+    <t>13.05° N / 77.51° E</t>
+  </si>
+  <si>
+    <t>iPlanet Vidyaranyapura</t>
+  </si>
+  <si>
+    <t>VID 1</t>
+  </si>
+  <si>
+    <t>HMT Layout 4th Block</t>
+  </si>
+  <si>
+    <t>Near TVS</t>
+  </si>
+  <si>
+    <t>No. 600, Ground Floor, Vidyaranyapura Main Road, HMT Layout 4th Block, Bengaluru – 560097.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Vidyaranyapura+Main+Road+Bengaluru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.08° N / 77.56° E </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gujarat </t>
+  </si>
+  <si>
+    <t>VAD 1</t>
+  </si>
+  <si>
+    <t>Shree Siddeshwar Havelock</t>
+  </si>
+  <si>
+    <t>Shop No. 3, Ground Floor, Shree Siddeshwar Havelock, Sama–Savli Road, Vemali, Vadodara, Gujarat – 390024.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Shree+Siddeshwar+Havelock+Vemali+Vadodara</t>
+  </si>
+  <si>
+    <t>22.3514° N / 73.2005° E</t>
+  </si>
+  <si>
+    <t>Opposite Bansal Mall, on Sama–Savli Road,</t>
+  </si>
+  <si>
+    <t>iPlanet Vadodara</t>
+  </si>
+  <si>
+    <t>iPlanet Seawoods Grand Central Mall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWD 1 </t>
+  </si>
+  <si>
+    <t>Seawoods Station Road</t>
+  </si>
+  <si>
+    <t>Seawoods Grand Central Mall, near Vaya Store.</t>
+  </si>
+  <si>
+    <t>UG 47, Seawoods Grand Central Mall, Seawoods Station Road, Sector 28, Nerul East, Navi Mumbai – 400706.</t>
+  </si>
+  <si>
+    <t>19.02° N / 73.02° E</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Seawoods+Grand+Central+Mall+Navi+Mumbai</t>
+  </si>
+  <si>
+    <t>iPlanet Inorbit Mall, Vashi</t>
+  </si>
+  <si>
+    <t>VAS 1</t>
+  </si>
+  <si>
+    <t>Inorbit Mall, near Vashi railway station.</t>
+  </si>
+  <si>
+    <t>Palm Beach Road</t>
+  </si>
+  <si>
+    <t>norbit Mall, Palm Beach Road, Sector 30A, Vashi, Navi Mumbai – 400703.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Inorbit+Mall+Vashi</t>
+  </si>
+  <si>
+    <t>19.06° N / 72.99° E</t>
+  </si>
+  <si>
+    <t>iPlanet Orion Mall, Panvel</t>
+  </si>
+  <si>
+    <t>PAN 1</t>
+  </si>
+  <si>
+    <t>Shop G16, Orion Mall, Forest Colony Road, Panvel, Navi Mumbai region – 410206.</t>
+  </si>
+  <si>
+    <t>Orion Mall, near Barbeque Nation.</t>
+  </si>
+  <si>
+    <t>Forest Colony Road</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Orion+Mall+Panvel</t>
+  </si>
+  <si>
+    <t>18.99° N / 73.12° E</t>
+  </si>
+  <si>
+    <t>iPlanet Prabhadevi</t>
+  </si>
+  <si>
+    <t>PDV 1</t>
+  </si>
+  <si>
+    <t>Appasaheb Marathe Marg</t>
+  </si>
+  <si>
+    <t>Opposite Mercedes-Benz showroom</t>
+  </si>
+  <si>
+    <t>No. 5, Jayant Apartments, Appasaheb Marathe Marg, Century Bazaar, Prabhadevi, Mumbai – 400025.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Prabhadevi+Jayant+Apartments+Mumbai</t>
+  </si>
+  <si>
+    <t>19.014° N / 72.829° E</t>
+  </si>
+  <si>
+    <t>iPlanet Tardeo</t>
+  </si>
+  <si>
+    <t>KEM 1</t>
+  </si>
+  <si>
+    <t>Hughes Road / N. S. Patkar Marg</t>
+  </si>
+  <si>
+    <t>Near DBS Bank, Tardeo.</t>
+  </si>
+  <si>
+    <t>18.97° N / 72.81° E</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Tardeo+Hughes+Road+Mumbai</t>
+  </si>
+  <si>
+    <t>No. 13, Ground Floor, Hughes Road / N. S. Patkar Marg, near DBS Bank, Tardeo, Mumbai – 400007.</t>
+  </si>
+  <si>
+    <t>iPlanet Khar West</t>
+  </si>
+  <si>
+    <t>LNK 1</t>
+  </si>
+  <si>
+    <t>Near Sangeeta Boochra</t>
+  </si>
+  <si>
+    <t>Linking Road</t>
+  </si>
+  <si>
+    <t>G27, Ground Floor, Linking Road, Khar West, Mumbai – 400052.</t>
+  </si>
+  <si>
+    <t>19.07° N / 72.83° E</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Khar+West+Linking+Road+Mumbai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kerala </t>
+  </si>
+  <si>
+    <t>Latitude &amp; Longitude</t>
+  </si>
+  <si>
+    <t>iPlanet Andheri West</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADH 1 </t>
+  </si>
+  <si>
+    <t>Parsi Colony</t>
+  </si>
+  <si>
+    <t>Zee Manu Bharti building, on S.V. Road</t>
+  </si>
+  <si>
+    <t>No. 1, Ground Floor, Zee Manu Bharti, Swami Vivekanand Road, Parsi Colony, Andheri West, Mumbai – 400056.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Andheri+West+Zee+Manu+Bharti+Mumbai</t>
+  </si>
+  <si>
+    <t>19.12° N / 72.84° E</t>
+  </si>
+  <si>
+    <t>iPlanet Powai</t>
+  </si>
+  <si>
+    <t>POW 1</t>
+  </si>
+  <si>
+    <t>Opposite D-Mart</t>
+  </si>
+  <si>
+    <t>Hiranandani Gardens</t>
+  </si>
+  <si>
+    <t>G12, Ground Floor, Ventura Building, Central Avenue, Hiranandani Gardens, Powai, Mumbai – 400076</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Powai+Ventura+Building+Mumbai</t>
+  </si>
+  <si>
+    <t>19.12° N / 72.91° E</t>
+  </si>
+  <si>
+    <t>iPlanet The Walk</t>
+  </si>
+  <si>
+    <t>WAK1</t>
+  </si>
+  <si>
+    <t>The Walk Mall, Hiranandani Estate</t>
+  </si>
+  <si>
+    <t>S10, The Walk, Hiranandani Estate Road, Hiranandani Estate, Thane West, Maharashtra – 400607</t>
+  </si>
+  <si>
+    <t>Hiranandani Estate Road</t>
+  </si>
+  <si>
+    <t>19.254972 / 72.984596</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+The+Walk+Hiranandani+Estate+Thane</t>
+  </si>
+  <si>
+    <t>iPlanet Naupada</t>
+  </si>
+  <si>
+    <t>NPD 1</t>
+  </si>
+  <si>
+    <t>Shop No. 1–2, Ground Floor, Rajesh CHS, Ram Maruti Road, Panch Pakhdi, Thane West – 400602.</t>
+  </si>
+  <si>
+    <t>Opposite SIB Bank, Ram Maruti Road</t>
+  </si>
+  <si>
+    <t>Panch Pakhdi</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Panch+Pakhdi+Ram+Maruti+Road+Thane</t>
+  </si>
+  <si>
+    <t>19.19° N / 72.97° E</t>
+  </si>
+  <si>
+    <t>iPlanet Viviana Mall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VVT 1 </t>
+  </si>
+  <si>
+    <t>Viviana Mall, Eastern Express Highway</t>
+  </si>
+  <si>
+    <t>Near Jupiter Hospital, inside Viviana Mall</t>
+  </si>
+  <si>
+    <t>Shop No. 62, Ground Floor, Viviana Mall, Eastern Express Highway, Thane West, Maharashtra – 400606.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Viviana+Mall+Thane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19.21° N, 72.97° E </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maharastra / Mumbai </t>
+  </si>
+  <si>
+    <t>Maharastra / Thane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maharastra / Satara </t>
+  </si>
+  <si>
+    <t>STR 1</t>
+  </si>
+  <si>
+    <t>Shop No. 4 &amp; 5, Upper Ground Floor, The Ahilya, Suryawanshi Colony, Sadar Bazar, Satara, Maharashtra – 415002</t>
+  </si>
+  <si>
+    <t>The Ahilya building, Suryawanshi Colony</t>
+  </si>
+  <si>
+    <t>Sadar Bazar</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+The+Ahilya+Sadar+Bazar+Satara</t>
+  </si>
+  <si>
+    <t>17.69° N / 74.01° E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iPlanet Satara </t>
+  </si>
+  <si>
+    <t xml:space="preserve">iPlanet Sangli </t>
+  </si>
+  <si>
+    <t>Ground Floor, Platinum Plaza, Miraj Road, Vijaynagar, Sangli Miraj Kupwad, Maharashtra – 416414.</t>
+  </si>
+  <si>
+    <t>Platinum Plaza on Miraj Road, Vijaynagar</t>
+  </si>
+  <si>
+    <t>Miraj Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maharastra / Sangli </t>
+  </si>
+  <si>
+    <t>MRJ 1</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Platinum+Plaza+Miraj+Road+Vijaynagar+Sangli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.85° N / 74.57° E </t>
+  </si>
+  <si>
+    <t>AP / TG</t>
+  </si>
+  <si>
+    <t>iPlanet Guntur</t>
+  </si>
+  <si>
+    <t>GTR 1</t>
+  </si>
+  <si>
+    <t>Brodipet</t>
+  </si>
+  <si>
+    <t>Near Grand Nagarjuna Hotel</t>
+  </si>
+  <si>
+    <t>Shop No. 1, Ground Floor, Beckker Compound, Brodipet Main Road, Brodipet, Guntur, Andhra Pradesh – 522002.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Beckker+Compound+Brodipet+Guntur</t>
+  </si>
+  <si>
+    <t>16.30° N / 80.44° E</t>
+  </si>
+  <si>
+    <t>iPlanet Tirupati</t>
+  </si>
+  <si>
+    <t>TPT 1</t>
+  </si>
+  <si>
+    <t>Avilali</t>
+  </si>
+  <si>
+    <t>Ground Floor, No. 166, Air Bypass Road, near Puma Store, New Balaji Colony, Avilali, Tirupati, Andhra Pradesh – 517502.</t>
+  </si>
+  <si>
+    <t>Near Puma Store, Air Bypass Road</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+166+Air+Bypass+Road+near+Puma+Store+Tirupati</t>
+  </si>
+  <si>
+    <t>13.62° N / 79.42° E</t>
+  </si>
+  <si>
+    <t>iPlanet Ongole</t>
+  </si>
+  <si>
+    <t>ONG 1</t>
+  </si>
+  <si>
+    <t>Trunk Road</t>
+  </si>
+  <si>
+    <t>Beside Axis Bank, Ravi Complex</t>
+  </si>
+  <si>
+    <t>No. 37/1/347, Ravi Complex, Trunk Road, Gadiyaram Vari Veedhi, Bandla Metla, Ongole, Andhra Pradesh – 523001.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Ravi+Complex+Trunk+Road+Ongole</t>
+  </si>
+  <si>
+    <t>15.50° N / 80.05° E</t>
+  </si>
+  <si>
+    <t>iPlanet Nalgonda</t>
+  </si>
+  <si>
+    <t>NGD 1</t>
+  </si>
+  <si>
+    <t>Opposite More Super Market, Hotel Siddhartha Complex.</t>
+  </si>
+  <si>
+    <t>Hyderabad Road, Sri Lakshmi Nagar Colony</t>
+  </si>
+  <si>
+    <t>Ground Floor, Hotel Siddhartha Complex, No. 6/2/562, Hyderabad Road, Sri Lakshmi Nagar Colony, Nalgonda, Telangana – 508001.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Hotel+Siddhartha+Complex+opposite+More+Super+Market+Nalgonda</t>
+  </si>
+  <si>
+    <t>17.05° N / 79.27° E</t>
+  </si>
+  <si>
+    <t>iPlanet Miryalaguda</t>
+  </si>
+  <si>
+    <t>MGD 1</t>
+  </si>
+  <si>
+    <t>Opposite GV Mall, Sagar Road</t>
+  </si>
+  <si>
+    <t>Hanumanpet</t>
+  </si>
+  <si>
+    <t>No. 18/1638, Sagar Road, Hanumanpet, Miryalaguda, Telangana – 508207.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+opposite+GV+Mall+Sagar+Road+Miryalaguda</t>
+  </si>
+  <si>
+    <t>16.87° N / 79.57° E</t>
+  </si>
+  <si>
+    <t>iPlanet Mancherial</t>
+  </si>
+  <si>
+    <t>MAN 1</t>
+  </si>
+  <si>
+    <t>Opposite Jio Petrol Bunk, Srisri Nagar,</t>
+  </si>
+  <si>
+    <t>Mancherial Road</t>
+  </si>
+  <si>
+    <t>No. 2269, Mancherial Road, Srisri Nagar, Mancherial, Telangana – 504208.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+2269+Mancherial+Road+opposite+Jio+Petrol+Bunk+Srisri+Nagar</t>
+  </si>
+  <si>
+    <t>19.0° N / 79.5° E</t>
+  </si>
+  <si>
+    <t>iPlanet Nizamabad</t>
+  </si>
+  <si>
+    <t>NZD 1</t>
+  </si>
+  <si>
+    <t>Opposite Hotel Midtown, Pragathi Nagar</t>
+  </si>
+  <si>
+    <t>Pragathi Nagar</t>
+  </si>
+  <si>
+    <t>No. 5-6-574 &amp; 573, Hyderabad Road, Pragathi Nagar, Nizamabad, Telangana – 503003.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+opposite+Hotel+Midtown+Pragathi+Nagar+Nizamabad</t>
+  </si>
+  <si>
+    <t>iPlanet Chanda Nagar</t>
+  </si>
+  <si>
+    <t>CDN 1</t>
+  </si>
+  <si>
+    <t>Opposite PRK Hospitals</t>
+  </si>
+  <si>
+    <t>Gouthami Nagar Colony, Jawahar Colony</t>
+  </si>
+  <si>
+    <t>Plot No. 4, No. 2-6-1/1, Service Road, Gouthami Nagar Colony, Jawahar Colony, Chanda Nagar, Hyderabad, Telangana – 502032.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+opposite+PRK+Hospitals+Chanda+Nagar+Hyderabad</t>
+  </si>
+  <si>
+    <t>18.67° N / 78.10° E</t>
+  </si>
+  <si>
+    <t>17.49° N / 78.33° E</t>
+  </si>
+  <si>
+    <t>iPlanet Kokapet One Mall</t>
+  </si>
+  <si>
+    <t>KOK 1</t>
+  </si>
+  <si>
+    <t>Kokapet One Mall</t>
+  </si>
+  <si>
+    <t>Gandipet Main Road</t>
+  </si>
+  <si>
+    <t>No. 11-5/3 &amp; 11-5/103, Kokapet One Mall, Gandipet Main Road, Kokapet, Narsingi, Hyderabad – 500075.</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Kokapet+One+Mall+Hyderabad</t>
+  </si>
+  <si>
+    <t>17.39° N / 78.35° E</t>
+  </si>
+  <si>
+    <t>iPlanet Vizag</t>
+  </si>
+  <si>
+    <t>VIZ 1</t>
+  </si>
+  <si>
+    <t>Inorbit Mall, Kailasapuram</t>
+  </si>
+  <si>
+    <t>No. 74 A, Upper Ground Floor, Inorbit Mall, Main Road, Zone-Z8, Kailasapuram, Visakhapatnam, Andhra Pradesh – 530024.</t>
+  </si>
+  <si>
+    <t>Zone-Z8, Kailasapuram</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Inorbit+Mall+Kailasapuram+Visakhapatnam</t>
+  </si>
+  <si>
+    <t>17.742539° N  / 83.297420° E</t>
+  </si>
+  <si>
+    <t>iPlanet Kakinada</t>
+  </si>
+  <si>
+    <t>KAK 1</t>
+  </si>
+  <si>
+    <t>82° East SRMT Mall &amp; Multiplex</t>
+  </si>
+  <si>
+    <t>Pithapuram–Kakinada Road</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Shop No. 10, 4-21, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>82° East SRMT Mall &amp; Multiplex</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, Pithapuram–Kakinada Road, Lalitha Nagar, Ramanayyapeta, Kakinada – 533005</t>
+    </r>
+  </si>
+  <si>
+    <t>16.989° N / 82.247° E</t>
+  </si>
+  <si>
+    <t>https://share.google/vHKCJajHKpfo28vaA</t>
+  </si>
+  <si>
+    <t>iPlanet Anantapur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANT 1 </t>
+  </si>
+  <si>
+    <t>Beside Balaji Travels</t>
+  </si>
+  <si>
+    <t>Kamalanagar</t>
+  </si>
+  <si>
+    <t>No. 15/775, Raju Road, Kamalanagar, Anantapur – 515001</t>
+  </si>
+  <si>
+    <t>14.6819° N / 77.6006° E</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=iPlanet+Kamalanagar+Anantapur+Raju+Road</t>
+  </si>
+  <si>
+    <t>iPlanet Eluru</t>
+  </si>
+  <si>
+    <t>ELR 1</t>
+  </si>
+  <si>
+    <t>RR Peta Main Road</t>
+  </si>
+  <si>
+    <t>Opp. Tanishq Jewellery, Powerpet</t>
+  </si>
+  <si>
+    <t>No. 23B-2-21, NSRK Complex, RR Peta Main Road, Powerpet, Eluru – 534002</t>
+  </si>
+  <si>
+    <t>16.7139 / 81.1053</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=16.7139,81.1053</t>
+  </si>
+  <si>
+    <t>iPlanet Dombivli</t>
+  </si>
+  <si>
+    <t>RNG 1</t>
+  </si>
+  <si>
+    <t>Kalyan Road, Trimurti Nagar</t>
+  </si>
+  <si>
+    <t>Ground Floor, Ambrin I, No. 1–3, Kalyan Road, Trimurti Nagar, Dombivli East, Kalyan – 421201</t>
+  </si>
+  <si>
+    <t>19.2183° N / 73.0867° E</t>
+  </si>
+  <si>
+    <t>https://www.google.com/maps/search/?api=1&amp;query=19.2183,73.0867</t>
+  </si>
+  <si>
+    <r>
+      <t>Near Pizza Hut</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1217,7 +2191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.5703125" customWidth="1"/>
@@ -1262,1243 +2236,2619 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
       <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
       </c>
       <c r="F2">
         <v>600017</v>
       </c>
       <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
       </c>
       <c r="F3">
         <v>600037</v>
       </c>
       <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>27</v>
       </c>
       <c r="F4">
         <v>600087</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>31</v>
-      </c>
-      <c r="I4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
         <v>33</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
         <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s">
-        <v>35</v>
       </c>
       <c r="F5">
         <v>600073</v>
       </c>
       <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
         <v>37</v>
       </c>
-      <c r="H5" t="s">
-        <v>36</v>
-      </c>
-      <c r="I5" t="s">
+      <c r="J5" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" t="s">
         <v>40</v>
       </c>
-      <c r="B6" t="s">
-        <v>41</v>
-      </c>
       <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
       <c r="E6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F6">
         <v>600097</v>
       </c>
       <c r="G6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" t="s">
         <v>42</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>43</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
         <v>46</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
         <v>47</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s">
-        <v>48</v>
       </c>
       <c r="F7">
         <v>600054</v>
       </c>
       <c r="G7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H7" t="s">
         <v>49</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>50</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
         <v>53</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
         <v>54</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>55</v>
-      </c>
-      <c r="E8" t="s">
-        <v>56</v>
       </c>
       <c r="F8">
         <v>641002</v>
       </c>
       <c r="G8" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>58</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" t="s">
         <v>61</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" t="s">
         <v>62</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s">
-        <v>63</v>
       </c>
       <c r="F9">
         <v>641012</v>
       </c>
       <c r="G9" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" t="s">
         <v>64</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>65</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" t="s">
         <v>68</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" t="s">
         <v>69</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E10" t="s">
-        <v>70</v>
       </c>
       <c r="F10">
         <v>641001</v>
       </c>
       <c r="G10" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" t="s">
         <v>71</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>72</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" t="s">
         <v>75</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
         <v>76</v>
-      </c>
-      <c r="C11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>55</v>
-      </c>
-      <c r="E11" t="s">
-        <v>77</v>
       </c>
       <c r="F11">
         <v>641045</v>
       </c>
       <c r="G11" t="s">
+        <v>77</v>
+      </c>
+      <c r="H11" t="s">
         <v>78</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>79</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B12" t="s">
         <v>82</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" t="s">
         <v>83</v>
-      </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" t="s">
-        <v>84</v>
       </c>
       <c r="F12">
         <v>641035</v>
       </c>
       <c r="G12" t="s">
+        <v>83</v>
+      </c>
+      <c r="H12" t="s">
+        <v>85</v>
+      </c>
+      <c r="I12" t="s">
         <v>84</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="I12" t="s">
-        <v>85</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" t="s">
         <v>88</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
         <v>89</v>
       </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>90</v>
-      </c>
-      <c r="E13" t="s">
-        <v>91</v>
       </c>
       <c r="F13">
         <v>625001</v>
       </c>
       <c r="G13" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" t="s">
         <v>92</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>93</v>
       </c>
-      <c r="I13" t="s">
-        <v>94</v>
-      </c>
       <c r="J13" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" t="s">
         <v>95</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" t="s">
         <v>96</v>
-      </c>
-      <c r="C14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s">
-        <v>90</v>
-      </c>
-      <c r="E14" t="s">
-        <v>97</v>
       </c>
       <c r="F14">
         <v>625016</v>
       </c>
       <c r="G14" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" t="s">
         <v>98</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>99</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" t="s">
         <v>102</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E15" t="s">
         <v>103</v>
-      </c>
-      <c r="C15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" t="s">
-        <v>90</v>
-      </c>
-      <c r="E15" t="s">
-        <v>104</v>
       </c>
       <c r="F15">
         <v>625020</v>
       </c>
       <c r="G15" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" t="s">
         <v>105</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>106</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" s="1" t="s">
         <v>107</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" t="s">
         <v>109</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
         <v>110</v>
       </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="E16" t="s">
         <v>111</v>
-      </c>
-      <c r="E16" t="s">
-        <v>112</v>
       </c>
       <c r="F16">
         <v>636004</v>
       </c>
       <c r="G16" t="s">
+        <v>112</v>
+      </c>
+      <c r="H16" t="s">
         <v>113</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>114</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="J16" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" t="s">
         <v>117</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>110</v>
+      </c>
+      <c r="E17" t="s">
         <v>118</v>
-      </c>
-      <c r="C17" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s">
-        <v>111</v>
-      </c>
-      <c r="E17" t="s">
-        <v>119</v>
       </c>
       <c r="F17">
         <v>636016</v>
       </c>
       <c r="G17" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" t="s">
         <v>120</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>121</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" t="s">
         <v>124</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
         <v>125</v>
       </c>
-      <c r="C18" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
         <v>126</v>
-      </c>
-      <c r="E18" t="s">
-        <v>127</v>
       </c>
       <c r="F18">
         <v>605001</v>
       </c>
       <c r="G18" t="s">
+        <v>127</v>
+      </c>
+      <c r="H18" t="s">
         <v>128</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>129</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>131</v>
+      </c>
+      <c r="B19" t="s">
         <v>132</v>
       </c>
-      <c r="B19" t="s">
-        <v>133</v>
-      </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D19" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F19">
         <v>605010</v>
       </c>
       <c r="G19" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H19" t="s">
+        <v>135</v>
+      </c>
+      <c r="I19" t="s">
         <v>136</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>138</v>
+      </c>
+      <c r="B20" t="s">
+        <v>146</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
         <v>139</v>
       </c>
-      <c r="B20" t="s">
-        <v>147</v>
-      </c>
-      <c r="C20" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" t="s">
-        <v>140</v>
-      </c>
       <c r="E20" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F20">
         <v>613007</v>
       </c>
       <c r="G20" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H20" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I20" t="s">
+        <v>143</v>
+      </c>
+      <c r="J20" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="J20" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B21" t="s">
+        <v>147</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
         <v>148</v>
       </c>
-      <c r="C21" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="E21" t="s">
         <v>149</v>
-      </c>
-      <c r="E21" t="s">
-        <v>150</v>
       </c>
       <c r="F21">
         <v>632006</v>
       </c>
       <c r="G21" t="s">
+        <v>150</v>
+      </c>
+      <c r="H21" t="s">
         <v>151</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>152</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>154</v>
+      </c>
+      <c r="B22" t="s">
         <v>155</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" t="s">
         <v>156</v>
-      </c>
-      <c r="C22" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" t="s">
-        <v>149</v>
-      </c>
-      <c r="E22" t="s">
-        <v>157</v>
       </c>
       <c r="F22">
         <v>632001</v>
       </c>
       <c r="G22" t="s">
+        <v>157</v>
+      </c>
+      <c r="H22" t="s">
         <v>158</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>159</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="J22" s="1" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B23" t="s">
+        <v>196</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
         <v>197</v>
       </c>
-      <c r="C23" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" t="s">
-        <v>198</v>
-      </c>
       <c r="E23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F23">
         <v>629001</v>
       </c>
       <c r="G23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H23" t="s">
+        <v>165</v>
+      </c>
+      <c r="I23" t="s">
+        <v>167</v>
+      </c>
+      <c r="J23" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="I23" t="s">
-        <v>168</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" t="s">
         <v>169</v>
       </c>
-      <c r="B24" t="s">
-        <v>170</v>
-      </c>
       <c r="C24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D24" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F24">
         <v>627002</v>
       </c>
       <c r="G24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H24" t="s">
+        <v>172</v>
+      </c>
+      <c r="I24" t="s">
         <v>173</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>175</v>
+      </c>
+      <c r="B25" t="s">
         <v>176</v>
       </c>
-      <c r="B25" t="s">
-        <v>177</v>
-      </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D25" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F25">
         <v>628002</v>
       </c>
       <c r="G25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H25" t="s">
+        <v>179</v>
+      </c>
+      <c r="I25" t="s">
+        <v>181</v>
+      </c>
+      <c r="J25" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="I25" t="s">
-        <v>182</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>182</v>
+      </c>
+      <c r="B26" t="s">
         <v>183</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
         <v>184</v>
       </c>
-      <c r="C26" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" t="s">
-        <v>185</v>
-      </c>
       <c r="E26" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F26">
         <v>620018</v>
       </c>
       <c r="G26" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H26" t="s">
+        <v>187</v>
+      </c>
+      <c r="I26" t="s">
         <v>188</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B27" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E27" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F27">
         <v>620019</v>
       </c>
       <c r="G27" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H27" t="s">
+        <v>192</v>
+      </c>
+      <c r="I27" t="s">
+        <v>195</v>
+      </c>
+      <c r="J27" s="1" t="s">
         <v>193</v>
-      </c>
-      <c r="I27" t="s">
-        <v>196</v>
-      </c>
-      <c r="J27" s="1" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B28" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E28" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F28">
         <v>641602</v>
       </c>
       <c r="G28" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H28" t="s">
+        <v>202</v>
+      </c>
+      <c r="I28" t="s">
+        <v>204</v>
+      </c>
+      <c r="J28" s="1" t="s">
         <v>203</v>
-      </c>
-      <c r="I28" t="s">
-        <v>205</v>
-      </c>
-      <c r="J28" s="1" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>277</v>
+      </c>
+      <c r="B29" t="s">
+        <v>278</v>
+      </c>
+      <c r="C29" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" t="s">
+        <v>162</v>
+      </c>
+      <c r="E29" t="s">
+        <v>281</v>
+      </c>
+      <c r="F29">
+        <v>636705</v>
+      </c>
+      <c r="G29" t="s">
         <v>280</v>
+      </c>
+      <c r="H29" t="s">
+        <v>279</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>279</v>
+        <v>206</v>
+      </c>
+      <c r="B30" t="s">
+        <v>209</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="s">
+        <v>439</v>
+      </c>
+      <c r="E30" t="s">
+        <v>208</v>
+      </c>
+      <c r="F30">
+        <v>670012</v>
+      </c>
+      <c r="G30" t="s">
+        <v>207</v>
+      </c>
+      <c r="H30" t="s">
+        <v>210</v>
+      </c>
+      <c r="I30" t="s">
+        <v>212</v>
+      </c>
+      <c r="J30" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="B31" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D31" t="s">
-        <v>211</v>
+        <v>439</v>
       </c>
       <c r="E31" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="F31">
-        <v>670012</v>
+        <v>682020</v>
       </c>
       <c r="G31" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="H31" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="I31" t="s">
-        <v>214</v>
-      </c>
-      <c r="J31" t="s">
-        <v>213</v>
+        <v>218</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="B32" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D32" t="s">
-        <v>211</v>
+        <v>439</v>
       </c>
       <c r="E32" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="F32">
-        <v>682020</v>
+        <v>686001</v>
       </c>
       <c r="G32" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="H32" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="I32" t="s">
-        <v>220</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>221</v>
+        <v>225</v>
+      </c>
+      <c r="J32" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="B33" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>211</v>
+        <v>439</v>
       </c>
       <c r="E33" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="F33">
-        <v>686001</v>
+        <v>678001</v>
       </c>
       <c r="G33" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H33" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="I33" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="J33" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B34" t="s">
+        <v>236</v>
+      </c>
+      <c r="C34" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" t="s">
+        <v>439</v>
+      </c>
+      <c r="E34" t="s">
         <v>237</v>
       </c>
-      <c r="C34" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" t="s">
-        <v>211</v>
-      </c>
-      <c r="E34" t="s">
-        <v>231</v>
-      </c>
       <c r="F34">
-        <v>678001</v>
+        <v>695001</v>
       </c>
       <c r="G34" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="H34" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="I34" t="s">
-        <v>233</v>
-      </c>
-      <c r="J34" t="s">
-        <v>234</v>
+        <v>240</v>
+      </c>
+      <c r="J34" s="1" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B35" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>211</v>
+        <v>439</v>
       </c>
       <c r="E35" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="F35">
-        <v>695001</v>
+        <v>695024</v>
       </c>
       <c r="G35" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="H35" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I35" t="s">
-        <v>242</v>
-      </c>
-      <c r="J35" s="1" t="s">
-        <v>241</v>
+        <v>245</v>
+      </c>
+      <c r="J35" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="B36" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D36" t="s">
-        <v>211</v>
+        <v>249</v>
       </c>
       <c r="E36" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F36">
-        <v>695024</v>
+        <v>575001</v>
       </c>
       <c r="G36" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="H36" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="I36" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="J36" t="s">
-        <v>248</v>
+        <v>254</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>255</v>
+      </c>
+      <c r="B37" t="s">
+        <v>256</v>
+      </c>
+      <c r="C37" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" t="s">
+        <v>249</v>
+      </c>
+      <c r="E37" t="s">
+        <v>258</v>
+      </c>
+      <c r="F37">
+        <v>575001</v>
+      </c>
+      <c r="G37" t="s">
+        <v>257</v>
+      </c>
+      <c r="H37" t="s">
+        <v>260</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="J37" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>262</v>
+      </c>
+      <c r="B38" t="s">
+        <v>265</v>
+      </c>
+      <c r="C38" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" t="s">
         <v>249</v>
       </c>
-      <c r="B38" t="s">
-        <v>250</v>
-      </c>
-      <c r="C38" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" t="s">
-        <v>251</v>
-      </c>
       <c r="E38" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="F38">
-        <v>575001</v>
+        <v>576104</v>
       </c>
       <c r="G38" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="H38" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="I38" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="J38" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="B39" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="E39" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="F39">
-        <v>575001</v>
+        <v>560038</v>
       </c>
       <c r="G39" t="s">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="H39" t="s">
-        <v>262</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>263</v>
+        <v>274</v>
+      </c>
+      <c r="I39" t="s">
+        <v>275</v>
       </c>
       <c r="J39" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="B40" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
       <c r="C40" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D40" t="s">
-        <v>251</v>
+        <v>271</v>
       </c>
       <c r="E40" t="s">
-        <v>266</v>
+        <v>287</v>
       </c>
       <c r="F40">
-        <v>576104</v>
+        <v>560048</v>
       </c>
       <c r="G40" t="s">
-        <v>265</v>
+        <v>286</v>
       </c>
       <c r="H40" t="s">
-        <v>268</v>
-      </c>
-      <c r="I40" t="s">
-        <v>269</v>
-      </c>
-      <c r="J40" t="s">
-        <v>270</v>
+        <v>288</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="J40" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>291</v>
+      </c>
+      <c r="B41" t="s">
+        <v>292</v>
+      </c>
+      <c r="C41" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" t="s">
+        <v>271</v>
+      </c>
+      <c r="E41" t="s">
+        <v>308</v>
+      </c>
+      <c r="F41">
+        <v>560048</v>
+      </c>
+      <c r="G41" t="s">
+        <v>293</v>
+      </c>
+      <c r="H41" t="s">
+        <v>309</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="J41" t="s">
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>295</v>
+      </c>
+      <c r="B42" t="s">
+        <v>294</v>
+      </c>
+      <c r="C42" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" t="s">
         <v>271</v>
       </c>
-      <c r="B42" t="s">
-        <v>272</v>
-      </c>
-      <c r="C42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" t="s">
-        <v>273</v>
-      </c>
       <c r="E42" t="s">
-        <v>274</v>
+        <v>296</v>
       </c>
       <c r="F42">
-        <v>560038</v>
+        <v>560043</v>
       </c>
       <c r="G42" t="s">
-        <v>275</v>
+        <v>297</v>
       </c>
       <c r="H42" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
       <c r="I42" t="s">
-        <v>277</v>
+        <v>299</v>
       </c>
       <c r="J42" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>301</v>
+      </c>
+      <c r="B43" t="s">
+        <v>302</v>
+      </c>
+      <c r="C43" t="s">
+        <v>11</v>
+      </c>
       <c r="D43" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E43" t="s">
+        <v>304</v>
+      </c>
+      <c r="F43">
+        <v>560077</v>
+      </c>
+      <c r="G43" t="s">
+        <v>303</v>
+      </c>
+      <c r="H43" t="s">
+        <v>305</v>
+      </c>
+      <c r="I43" t="s">
+        <v>306</v>
+      </c>
+      <c r="J43" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>312</v>
+      </c>
+      <c r="B44" t="s">
+        <v>313</v>
+      </c>
+      <c r="C44" t="s">
+        <v>11</v>
+      </c>
       <c r="D44" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E44" t="s">
+        <v>315</v>
+      </c>
+      <c r="F44">
+        <v>560092</v>
+      </c>
+      <c r="G44" t="s">
+        <v>314</v>
+      </c>
+      <c r="H44" t="s">
+        <v>316</v>
+      </c>
+      <c r="I44" t="s">
+        <v>317</v>
+      </c>
+      <c r="J44" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>319</v>
+      </c>
+      <c r="B45" t="s">
+        <v>320</v>
+      </c>
+      <c r="C45" t="s">
+        <v>11</v>
+      </c>
       <c r="D45" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E45" t="s">
+        <v>322</v>
+      </c>
+      <c r="F45">
+        <v>560094</v>
+      </c>
+      <c r="G45" t="s">
+        <v>321</v>
+      </c>
+      <c r="H45" t="s">
+        <v>323</v>
+      </c>
+      <c r="I45" t="s">
+        <v>324</v>
+      </c>
+      <c r="J45" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>326</v>
+      </c>
+      <c r="B46" t="s">
+        <v>327</v>
+      </c>
+      <c r="C46" t="s">
+        <v>11</v>
+      </c>
       <c r="D46" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E46" t="s">
+        <v>328</v>
+      </c>
+      <c r="F46">
+        <v>560064</v>
+      </c>
+      <c r="G46" t="s">
+        <v>329</v>
+      </c>
+      <c r="H46" t="s">
+        <v>330</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>333</v>
+      </c>
+      <c r="B47" t="s">
+        <v>334</v>
+      </c>
+      <c r="C47" t="s">
+        <v>11</v>
+      </c>
       <c r="D47" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E47" t="s">
+        <v>335</v>
+      </c>
+      <c r="F47">
+        <v>560078</v>
+      </c>
+      <c r="G47" t="s">
+        <v>336</v>
+      </c>
+      <c r="H47" t="s">
+        <v>337</v>
+      </c>
+      <c r="I47" t="s">
+        <v>338</v>
+      </c>
+      <c r="J47" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>354</v>
+      </c>
+      <c r="B48" t="s">
+        <v>340</v>
+      </c>
+      <c r="C48" t="s">
+        <v>11</v>
+      </c>
       <c r="D48" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+        <v>271</v>
+      </c>
+      <c r="E48" t="s">
+        <v>342</v>
+      </c>
+      <c r="F48">
+        <v>560011</v>
+      </c>
+      <c r="G48" t="s">
+        <v>341</v>
+      </c>
+      <c r="H48" t="s">
+        <v>343</v>
+      </c>
+      <c r="I48" t="s">
+        <v>344</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>355</v>
+      </c>
+      <c r="B49" t="s">
+        <v>346</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
       <c r="D49" t="s">
-        <v>273</v>
+        <v>271</v>
+      </c>
+      <c r="E49" t="s">
+        <v>347</v>
+      </c>
+      <c r="F49">
+        <v>560076</v>
+      </c>
+      <c r="G49" t="s">
+        <v>348</v>
+      </c>
+      <c r="H49" t="s">
+        <v>349</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="J49" s="1" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>353</v>
+      </c>
+      <c r="B50" t="s">
+        <v>352</v>
+      </c>
+      <c r="C50" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" t="s">
+        <v>271</v>
+      </c>
+      <c r="E50" t="s">
+        <v>356</v>
+      </c>
+      <c r="F50">
+        <v>560085</v>
+      </c>
+      <c r="G50" t="s">
+        <v>358</v>
+      </c>
+      <c r="H50" t="s">
+        <v>357</v>
+      </c>
+      <c r="I50" t="s">
+        <v>359</v>
+      </c>
+      <c r="J50" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>361</v>
+      </c>
+      <c r="B51" t="s">
+        <v>362</v>
+      </c>
+      <c r="C51" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" t="s">
+        <v>271</v>
+      </c>
+      <c r="E51" t="s">
+        <v>365</v>
+      </c>
+      <c r="F51">
+        <v>560056</v>
+      </c>
+      <c r="G51" t="s">
+        <v>363</v>
+      </c>
+      <c r="H51" t="s">
+        <v>364</v>
+      </c>
+      <c r="I51" t="s">
+        <v>366</v>
+      </c>
+      <c r="J51" s="1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>368</v>
+      </c>
+      <c r="B52" t="s">
+        <v>369</v>
+      </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" t="s">
+        <v>271</v>
+      </c>
+      <c r="E52" t="s">
+        <v>371</v>
+      </c>
+      <c r="F52">
+        <v>560062</v>
+      </c>
+      <c r="G52" t="s">
+        <v>370</v>
+      </c>
+      <c r="H52" t="s">
+        <v>372</v>
+      </c>
+      <c r="I52" t="s">
+        <v>373</v>
+      </c>
+      <c r="J52" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>375</v>
+      </c>
+      <c r="B53" t="s">
+        <v>376</v>
+      </c>
+      <c r="C53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D53" t="s">
+        <v>271</v>
+      </c>
+      <c r="E53" t="s">
+        <v>377</v>
+      </c>
+      <c r="F53">
+        <v>560073</v>
+      </c>
+      <c r="G53" t="s">
+        <v>378</v>
+      </c>
+      <c r="H53" t="s">
+        <v>379</v>
+      </c>
+      <c r="I53" t="s">
+        <v>380</v>
+      </c>
+      <c r="J53" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>382</v>
+      </c>
+      <c r="B54" t="s">
+        <v>383</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" t="s">
+        <v>271</v>
+      </c>
+      <c r="E54" t="s">
+        <v>384</v>
+      </c>
+      <c r="F54">
+        <v>560097</v>
+      </c>
+      <c r="G54" t="s">
+        <v>385</v>
+      </c>
+      <c r="H54" t="s">
+        <v>386</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="J54" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>396</v>
+      </c>
+      <c r="B55" t="s">
+        <v>390</v>
+      </c>
+      <c r="C55" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" t="s">
+        <v>389</v>
+      </c>
+      <c r="E55" t="s">
+        <v>391</v>
+      </c>
+      <c r="F55">
+        <v>390024</v>
+      </c>
+      <c r="G55" t="s">
+        <v>395</v>
+      </c>
+      <c r="H55" t="s">
+        <v>392</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="J55" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>397</v>
+      </c>
+      <c r="B56" t="s">
+        <v>398</v>
+      </c>
+      <c r="C56" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" t="s">
+        <v>476</v>
+      </c>
+      <c r="E56" t="s">
+        <v>399</v>
+      </c>
+      <c r="F56">
+        <v>400706</v>
+      </c>
+      <c r="G56" t="s">
+        <v>400</v>
+      </c>
+      <c r="H56" t="s">
+        <v>401</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="J56" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>404</v>
+      </c>
+      <c r="B57" t="s">
+        <v>405</v>
+      </c>
+      <c r="C57" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" t="s">
+        <v>476</v>
+      </c>
+      <c r="E57" t="s">
+        <v>407</v>
+      </c>
+      <c r="F57">
+        <v>400703</v>
+      </c>
+      <c r="G57" t="s">
+        <v>406</v>
+      </c>
+      <c r="H57" t="s">
+        <v>408</v>
+      </c>
+      <c r="I57" t="s">
+        <v>409</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>411</v>
+      </c>
+      <c r="B58" t="s">
+        <v>412</v>
+      </c>
+      <c r="C58" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" t="s">
+        <v>476</v>
+      </c>
+      <c r="E58" t="s">
+        <v>415</v>
+      </c>
+      <c r="F58">
+        <v>410206</v>
+      </c>
+      <c r="G58" t="s">
+        <v>414</v>
+      </c>
+      <c r="H58" t="s">
+        <v>413</v>
+      </c>
+      <c r="I58" t="s">
+        <v>416</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>418</v>
+      </c>
+      <c r="B59" t="s">
+        <v>419</v>
+      </c>
+      <c r="C59" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" t="s">
+        <v>476</v>
+      </c>
+      <c r="E59" t="s">
+        <v>420</v>
+      </c>
+      <c r="F59">
+        <v>400025</v>
+      </c>
+      <c r="G59" t="s">
+        <v>421</v>
+      </c>
+      <c r="H59" t="s">
+        <v>422</v>
+      </c>
+      <c r="I59" t="s">
+        <v>423</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>425</v>
+      </c>
+      <c r="B60" t="s">
+        <v>426</v>
+      </c>
+      <c r="C60" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" t="s">
+        <v>476</v>
+      </c>
+      <c r="E60" t="s">
+        <v>427</v>
+      </c>
+      <c r="F60">
+        <v>400007</v>
+      </c>
+      <c r="G60" t="s">
+        <v>428</v>
+      </c>
+      <c r="H60" t="s">
+        <v>431</v>
+      </c>
+      <c r="I60" t="s">
+        <v>430</v>
+      </c>
+      <c r="J60" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>432</v>
+      </c>
+      <c r="B61" t="s">
+        <v>433</v>
+      </c>
+      <c r="C61" t="s">
+        <v>11</v>
+      </c>
+      <c r="D61" t="s">
+        <v>476</v>
+      </c>
+      <c r="E61" t="s">
+        <v>435</v>
+      </c>
+      <c r="F61">
+        <v>400052</v>
+      </c>
+      <c r="G61" t="s">
+        <v>434</v>
+      </c>
+      <c r="H61" t="s">
+        <v>436</v>
+      </c>
+      <c r="I61" t="s">
+        <v>438</v>
+      </c>
+      <c r="J61" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>441</v>
+      </c>
+      <c r="B62" t="s">
+        <v>442</v>
+      </c>
+      <c r="C62" t="s">
+        <v>11</v>
+      </c>
+      <c r="D62" t="s">
+        <v>476</v>
+      </c>
+      <c r="E62" t="s">
+        <v>443</v>
+      </c>
+      <c r="F62">
+        <v>400056</v>
+      </c>
+      <c r="G62" t="s">
+        <v>444</v>
+      </c>
+      <c r="H62" t="s">
+        <v>445</v>
+      </c>
+      <c r="I62" t="s">
+        <v>446</v>
+      </c>
+      <c r="J62" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>448</v>
+      </c>
+      <c r="B63" t="s">
+        <v>449</v>
+      </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" t="s">
+        <v>476</v>
+      </c>
+      <c r="E63" t="s">
+        <v>451</v>
+      </c>
+      <c r="F63">
+        <v>400076</v>
+      </c>
+      <c r="G63" t="s">
+        <v>450</v>
+      </c>
+      <c r="H63" t="s">
+        <v>452</v>
+      </c>
+      <c r="I63" t="s">
+        <v>453</v>
+      </c>
+      <c r="J63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>455</v>
+      </c>
+      <c r="B64" t="s">
+        <v>456</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>477</v>
+      </c>
+      <c r="E64" t="s">
+        <v>457</v>
+      </c>
+      <c r="F64">
+        <v>400607</v>
+      </c>
+      <c r="G64" t="s">
+        <v>459</v>
+      </c>
+      <c r="H64" t="s">
+        <v>458</v>
+      </c>
+      <c r="I64" t="s">
+        <v>461</v>
+      </c>
+      <c r="J64" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>462</v>
+      </c>
+      <c r="B65" t="s">
+        <v>463</v>
+      </c>
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" t="s">
+        <v>477</v>
+      </c>
+      <c r="E65" t="s">
+        <v>466</v>
+      </c>
+      <c r="F65">
+        <v>400602</v>
+      </c>
+      <c r="G65" t="s">
+        <v>465</v>
+      </c>
+      <c r="H65" t="s">
+        <v>464</v>
+      </c>
+      <c r="I65" t="s">
+        <v>467</v>
+      </c>
+      <c r="J65" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>469</v>
+      </c>
+      <c r="B66" t="s">
+        <v>470</v>
+      </c>
+      <c r="C66" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" t="s">
+        <v>477</v>
+      </c>
+      <c r="E66" t="s">
+        <v>471</v>
+      </c>
+      <c r="F66">
+        <v>400606</v>
+      </c>
+      <c r="G66" t="s">
+        <v>472</v>
+      </c>
+      <c r="H66" t="s">
+        <v>473</v>
+      </c>
+      <c r="I66" t="s">
+        <v>474</v>
+      </c>
+      <c r="J66" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>586</v>
+      </c>
+      <c r="B67" t="s">
+        <v>587</v>
+      </c>
+      <c r="C67" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" t="s">
+        <v>476</v>
+      </c>
+      <c r="E67" t="s">
+        <v>588</v>
+      </c>
+      <c r="F67">
+        <v>421201</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="H67" t="s">
+        <v>589</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="J67" s="1" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>485</v>
+      </c>
+      <c r="B68" t="s">
+        <v>479</v>
+      </c>
+      <c r="C68" t="s">
+        <v>11</v>
+      </c>
+      <c r="D68" t="s">
+        <v>478</v>
+      </c>
+      <c r="E68" t="s">
+        <v>482</v>
+      </c>
+      <c r="F68">
+        <v>415002</v>
+      </c>
+      <c r="G68" t="s">
+        <v>481</v>
+      </c>
+      <c r="H68" t="s">
+        <v>480</v>
+      </c>
+      <c r="I68" t="s">
+        <v>483</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>486</v>
+      </c>
+      <c r="B69" t="s">
+        <v>491</v>
+      </c>
+      <c r="C69" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69" t="s">
+        <v>490</v>
+      </c>
+      <c r="E69" t="s">
+        <v>489</v>
+      </c>
+      <c r="F69">
+        <v>416414</v>
+      </c>
+      <c r="G69" t="s">
+        <v>488</v>
+      </c>
+      <c r="H69" t="s">
+        <v>487</v>
+      </c>
+      <c r="I69" t="s">
+        <v>492</v>
+      </c>
+      <c r="J69" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>495</v>
+      </c>
+      <c r="B70" t="s">
+        <v>496</v>
+      </c>
+      <c r="C70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" t="s">
+        <v>494</v>
+      </c>
+      <c r="E70" t="s">
+        <v>497</v>
+      </c>
+      <c r="F70">
+        <v>522002</v>
+      </c>
+      <c r="G70" t="s">
+        <v>498</v>
+      </c>
+      <c r="H70" t="s">
+        <v>499</v>
+      </c>
+      <c r="I70" t="s">
+        <v>500</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>502</v>
+      </c>
+      <c r="B71" t="s">
+        <v>503</v>
+      </c>
+      <c r="C71" t="s">
+        <v>11</v>
+      </c>
+      <c r="D71" t="s">
+        <v>494</v>
+      </c>
+      <c r="E71" t="s">
+        <v>504</v>
+      </c>
+      <c r="F71">
+        <v>517502</v>
+      </c>
+      <c r="G71" t="s">
+        <v>506</v>
+      </c>
+      <c r="H71" t="s">
+        <v>505</v>
+      </c>
+      <c r="I71" t="s">
+        <v>507</v>
+      </c>
+      <c r="J71" s="1" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>509</v>
+      </c>
+      <c r="B72" t="s">
+        <v>510</v>
+      </c>
+      <c r="C72" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" t="s">
+        <v>494</v>
+      </c>
+      <c r="E72" t="s">
+        <v>511</v>
+      </c>
+      <c r="F72">
+        <v>523001</v>
+      </c>
+      <c r="G72" t="s">
+        <v>512</v>
+      </c>
+      <c r="H72" t="s">
+        <v>513</v>
+      </c>
+      <c r="I72" t="s">
+        <v>514</v>
+      </c>
+      <c r="J72" s="1" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>516</v>
+      </c>
+      <c r="B73" t="s">
+        <v>517</v>
+      </c>
+      <c r="C73" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" t="s">
+        <v>494</v>
+      </c>
+      <c r="E73" t="s">
+        <v>519</v>
+      </c>
+      <c r="F73">
+        <v>508001</v>
+      </c>
+      <c r="G73" t="s">
+        <v>518</v>
+      </c>
+      <c r="H73" t="s">
+        <v>520</v>
+      </c>
+      <c r="I73" t="s">
+        <v>521</v>
+      </c>
+      <c r="J73" s="1" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>523</v>
+      </c>
+      <c r="B74" t="s">
+        <v>524</v>
+      </c>
+      <c r="C74" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" t="s">
+        <v>494</v>
+      </c>
+      <c r="E74" t="s">
+        <v>526</v>
+      </c>
+      <c r="F74">
+        <v>508207</v>
+      </c>
+      <c r="G74" t="s">
+        <v>525</v>
+      </c>
+      <c r="H74" t="s">
+        <v>527</v>
+      </c>
+      <c r="I74" t="s">
+        <v>528</v>
+      </c>
+      <c r="J74" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>530</v>
+      </c>
+      <c r="B75" t="s">
+        <v>531</v>
+      </c>
+      <c r="C75" t="s">
+        <v>11</v>
+      </c>
+      <c r="D75" t="s">
+        <v>494</v>
+      </c>
+      <c r="E75" t="s">
+        <v>533</v>
+      </c>
+      <c r="F75">
+        <v>504208</v>
+      </c>
+      <c r="G75" t="s">
+        <v>532</v>
+      </c>
+      <c r="H75" t="s">
+        <v>534</v>
+      </c>
+      <c r="I75" t="s">
+        <v>535</v>
+      </c>
+      <c r="J75" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>537</v>
+      </c>
+      <c r="B76" t="s">
+        <v>538</v>
+      </c>
+      <c r="C76" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" t="s">
+        <v>494</v>
+      </c>
+      <c r="E76" t="s">
+        <v>540</v>
+      </c>
+      <c r="F76">
+        <v>503003</v>
+      </c>
+      <c r="G76" t="s">
+        <v>539</v>
+      </c>
+      <c r="H76" t="s">
+        <v>541</v>
+      </c>
+      <c r="I76" t="s">
+        <v>542</v>
+      </c>
+      <c r="J76" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>543</v>
+      </c>
+      <c r="B77" t="s">
+        <v>544</v>
+      </c>
+      <c r="C77" t="s">
+        <v>11</v>
+      </c>
+      <c r="D77" t="s">
+        <v>494</v>
+      </c>
+      <c r="E77" t="s">
+        <v>546</v>
+      </c>
+      <c r="F77">
+        <v>502032</v>
+      </c>
+      <c r="G77" t="s">
+        <v>545</v>
+      </c>
+      <c r="H77" t="s">
+        <v>547</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="J77" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>551</v>
+      </c>
+      <c r="B78" t="s">
+        <v>552</v>
+      </c>
+      <c r="C78" t="s">
+        <v>11</v>
+      </c>
+      <c r="D78" t="s">
+        <v>494</v>
+      </c>
+      <c r="E78" t="s">
+        <v>554</v>
+      </c>
+      <c r="F78">
+        <v>500075</v>
+      </c>
+      <c r="G78" t="s">
+        <v>553</v>
+      </c>
+      <c r="H78" t="s">
+        <v>555</v>
+      </c>
+      <c r="I78" t="s">
+        <v>556</v>
+      </c>
+      <c r="J78" s="1" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>558</v>
+      </c>
+      <c r="B79" t="s">
+        <v>559</v>
+      </c>
+      <c r="C79" t="s">
+        <v>11</v>
+      </c>
+      <c r="D79" t="s">
+        <v>494</v>
+      </c>
+      <c r="E79" t="s">
+        <v>562</v>
+      </c>
+      <c r="F79">
+        <v>530024</v>
+      </c>
+      <c r="G79" t="s">
+        <v>560</v>
+      </c>
+      <c r="H79" t="s">
+        <v>561</v>
+      </c>
+      <c r="I79" t="s">
+        <v>563</v>
+      </c>
+      <c r="J79" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>565</v>
+      </c>
+      <c r="B80" t="s">
+        <v>566</v>
+      </c>
+      <c r="C80" t="s">
+        <v>11</v>
+      </c>
+      <c r="D80" t="s">
+        <v>494</v>
+      </c>
+      <c r="E80" t="s">
+        <v>568</v>
+      </c>
+      <c r="F80">
+        <v>533005</v>
+      </c>
+      <c r="G80" t="s">
+        <v>567</v>
+      </c>
+      <c r="H80" t="s">
+        <v>569</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>572</v>
+      </c>
+      <c r="B81" t="s">
+        <v>573</v>
+      </c>
+      <c r="C81" t="s">
+        <v>11</v>
+      </c>
+      <c r="D81" t="s">
+        <v>494</v>
+      </c>
+      <c r="E81" t="s">
+        <v>575</v>
+      </c>
+      <c r="F81">
+        <v>515001</v>
+      </c>
+      <c r="G81" t="s">
+        <v>574</v>
+      </c>
+      <c r="H81" t="s">
+        <v>576</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>578</v>
+      </c>
+      <c r="J81" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>579</v>
+      </c>
+      <c r="B82" t="s">
+        <v>580</v>
+      </c>
+      <c r="C82" t="s">
+        <v>11</v>
+      </c>
+      <c r="D82" t="s">
+        <v>494</v>
+      </c>
+      <c r="E82" t="s">
+        <v>581</v>
+      </c>
+      <c r="F82">
+        <v>534002</v>
+      </c>
+      <c r="G82" t="s">
+        <v>582</v>
+      </c>
+      <c r="H82" t="s">
+        <v>583</v>
+      </c>
+      <c r="I82" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="J82" s="1" t="s">
+        <v>584</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="I39" r:id="rId1"/>
+    <hyperlink ref="I37" r:id="rId1"/>
+    <hyperlink ref="I29" r:id="rId2"/>
+    <hyperlink ref="I40" r:id="rId3"/>
+    <hyperlink ref="I41" r:id="rId4"/>
+    <hyperlink ref="I46" r:id="rId5"/>
+    <hyperlink ref="I49" r:id="rId6"/>
+    <hyperlink ref="I54" r:id="rId7"/>
+    <hyperlink ref="I55" r:id="rId8"/>
+    <hyperlink ref="I56" r:id="rId9"/>
+    <hyperlink ref="I77" r:id="rId10"/>
+    <hyperlink ref="I80" r:id="rId11"/>
+    <hyperlink ref="I81" r:id="rId12"/>
+    <hyperlink ref="I82" r:id="rId13"/>
+    <hyperlink ref="I67" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>